<commit_message>
user on INTERNAL portal added
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_PATCH.xlsx
+++ b/src/main/resources/Program_Field_Values_PATCH.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91697267-8FEF-4FFE-A504-83490596D3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7870BE-835F-47EA-90A0-556A7D4AA69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticRecordProgramCreation" sheetId="39" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="152">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -401,9 +401,6 @@
     <t>Automation Direct Grant</t>
   </si>
   <si>
-    <t>Automation Program For Test</t>
-  </si>
-  <si>
     <t>Automation Program For Announcement</t>
   </si>
   <si>
@@ -425,9 +422,6 @@
     <t>Program Manager</t>
   </si>
   <si>
-    <t>GMS Administrator</t>
-  </si>
-  <si>
     <t>fieldAllocationlevel__c</t>
   </si>
   <si>
@@ -483,6 +477,24 @@
   </si>
   <si>
     <t>Objectives__c</t>
+  </si>
+  <si>
+    <t>Automation Runtime Internal Program</t>
+  </si>
+  <si>
+    <t>Type__c</t>
+  </si>
+  <si>
+    <t>PrimaryFundingOrganization__c</t>
+  </si>
+  <si>
+    <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>FocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -545,7 +557,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -562,6 +574,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1271,7 +1289,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C5">
         <v>300</v>
@@ -1377,7 +1395,7 @@
         <v>97</v>
       </c>
       <c r="C8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1521,10 +1539,10 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -1532,10 +1550,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1936,7 +1954,7 @@
         <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2024,10 +2042,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2035,10 +2053,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -2046,10 +2064,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -2097,85 +2115,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C2" t="s">
-        <v>120</v>
+      <c r="C2" s="8" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="A3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" t="s">
-        <v>128</v>
+      <c r="A4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
+      <c r="A5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
+      <c r="A6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
+      <c r="A7" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" tooltip="https://test7-internal.my.salesforce.com/00e0b000001fm3y" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{8D7FE799-8783-40F7-87C7-3B66C044DD34}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2204,10 +2225,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -2215,10 +2236,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -2226,7 +2247,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2536,10 +2557,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2572,7 +2593,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -2583,10 +2604,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -2605,7 +2626,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -2616,7 +2637,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C6">
         <v>10000</v>
@@ -2627,7 +2648,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -2638,7 +2659,7 @@
         <v>16</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C8">
         <v>10000</v>

</xml_diff>

<commit_message>
pagelayout classic tc update
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values_PATCH.xlsx
+++ b/src/main/resources/Program_Field_Values_PATCH.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2987F7-DF88-4F96-B652-EE42963446B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5893093B-D396-453F-9DB4-EA3EFA68D31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="19" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StaticRecordProgramCreation" sheetId="39" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="SiteVisitEdition_v" sheetId="35" r:id="rId19"/>
     <sheet name="GeneralReviewForm_v" sheetId="36" r:id="rId20"/>
     <sheet name="Contacts" sheetId="41" r:id="rId21"/>
+    <sheet name="ContactCreation" sheetId="43" r:id="rId22"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="169">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -496,6 +497,57 @@
   </si>
   <si>
     <t>Automation Program For Test</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>Automation Runtime Contact</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>AutomationManager@yopmail.com</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>SterlingUSA</t>
+  </si>
+  <si>
+    <t>MailingCity</t>
+  </si>
+  <si>
+    <t>State__c</t>
+  </si>
+  <si>
+    <t>MailingPostalCode</t>
+  </si>
+  <si>
+    <t>MailingCountry</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>MobilePhone</t>
+  </si>
+  <si>
+    <t>ProjectRole__c</t>
+  </si>
+  <si>
+    <t>fieldMailingStreet</t>
+  </si>
+  <si>
+    <t>MH</t>
   </si>
 </sst>
 </file>
@@ -558,7 +610,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -580,6 +632,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2208,6 +2263,144 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB8C3BA-E383-402A-AD87-FB992F14A5E1}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="21.90625" customWidth="1"/>
+    <col min="3" max="3" width="38.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" s="10">
+        <v>7856789209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10">
+        <v>20171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" xr:uid="{C8AC352D-35A2-405F-982E-3B7FAF90C7BD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E83D430-2DDF-4C96-A733-8F6A18593E6C}">
   <dimension ref="A1:C7"/>

</xml_diff>